<commit_message>
Keep the 68 districts the 2026-27 realignment dissolved
The index was built from today's district list, so a district that no longer
exists fell off the board entirely - District 121 among them. Toastmasters
listed 125-132 districts in each finished year and lists 94 today: 68 were
dissolved into a new 200-series.

The index is now the union of all six years. A dissolved district keeps its
finished years, which are the record of what its clubs did, and appears in the
selector under 'No longer a district' with the last year it was listed. It has
no open year, so #inyear is hidden and #gonedistrict says why rather than
letting a reader land in the in-year error path, which claims the data failed
to load.

An id that resolves to a different district now rewrites the URL to match, so
?d=121 can no longer sit in the bar beside a wordmark reading District 227.

162 districts, 26 MB, 972 fetches, zero contrast failures in both themes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/d/02/inyear.xlsx
+++ b/docs/d/02/inyear.xlsx
@@ -495,7 +495,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Program year 2026-2027. Dashboard snapshot 22-Sep-2026. Built 2026-09-23 09:04 PDT.</t>
+          <t>Program year 2026-2027. Dashboard snapshot 23-Sep-2026. Built 2026-09-23 23:13 PDT.</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Renewal dues on time - closes 2027-03-31 (189 days) - 92 clubs short</t>
+          <t xml:space="preserve">   Renewal dues on time - closes 2027-03-31 (189 days) - 90 clubs short</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2777,7 @@
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F21" s="6" t="n">
         <v>10</v>
@@ -2847,8 +2847,8 @@
       <c r="Y21" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="Z21" s="9" t="n">
-        <v>0</v>
+      <c r="Z21" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="AA21" s="10" t="n">
         <v>1</v>
@@ -6489,7 +6489,7 @@
         <v>0</v>
       </c>
       <c r="Q57" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R57" s="9" t="n">
         <v>0</v>
@@ -6546,7 +6546,7 @@
         </is>
       </c>
       <c r="E58" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F58" s="6" t="n">
         <v>10</v>
@@ -6598,8 +6598,8 @@
       <c r="S58" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="T58" s="9" t="n">
-        <v>0</v>
+      <c r="T58" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="U58" s="9" t="n">
         <v>0</v>
@@ -8588,13 +8588,13 @@
         </is>
       </c>
       <c r="I78" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J78" s="4" t="n">
         <v>11</v>
       </c>
       <c r="K78" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L78" s="8" t="inlineStr">
         <is>
@@ -8633,7 +8633,7 @@
         <v>0</v>
       </c>
       <c r="V78" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W78" s="9" t="n">
         <v>0</v>
@@ -14787,7 +14787,7 @@
         </is>
       </c>
       <c r="E139" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F139" s="6" t="n">
         <v>10</v>
@@ -14857,8 +14857,8 @@
       <c r="Y139" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="Z139" s="9" t="n">
-        <v>0</v>
+      <c r="Z139" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="AA139" s="10" t="n">
         <v>1</v>
@@ -21802,7 +21802,7 @@
         <v>4</v>
       </c>
       <c r="D6" t="n">
-        <v>1.5</v>
+        <v>1.75</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -22033,7 +22033,7 @@
         <v>5</v>
       </c>
       <c r="D13" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
@@ -22594,7 +22594,7 @@
         <v>6</v>
       </c>
       <c r="D30" t="n">
-        <v>0.83</v>
+        <v>1</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>

</xml_diff>